<commit_message>
Templates: generic names for brand sample rows in Teacher Budget Planner; regenerate xlsx
</commit_message>
<xml_diff>
--- a/templates/Teacher_Budget_Planner.xlsx
+++ b/templates/Teacher_Budget_Planner.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Monthly Budget" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Classroom Spending" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Summer Planner" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Salary Comparison" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Instructions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Budget" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classroom Spending" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summer Planner" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Salary Comparison" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -866,7 +866,7 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Subscriptions (Netflix, Spotify, etc.)</t>
+          <t>Subscriptions (streaming service, music subscription, etc.)</t>
         </is>
       </c>
       <c r="B21" s="6" t="n">
@@ -1042,7 +1042,7 @@
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>Expo markers (bulk)</t>
+          <t>Dry-erase markers (bulk)</t>
         </is>
       </c>
       <c r="C2" s="14" t="inlineStr">
@@ -1166,7 +1166,7 @@
       </c>
       <c r="G5" s="16" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Online retailer</t>
         </is>
       </c>
     </row>
@@ -1264,7 +1264,7 @@
       </c>
       <c r="G8" s="14" t="inlineStr">
         <is>
-          <t>Dollar Tree</t>
+          <t>Dollar store</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>Scholastic book order (class set)</t>
+          <t>Book order (class set)</t>
         </is>
       </c>
       <c r="C9" s="16" t="inlineStr">

</xml_diff>

<commit_message>
Templates: generic names for brand sample rows in Teacher Budget Planner; regenerate xlsx (#41)
Co-authored-by: asj412-cpu <asj412-cpu@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/templates/Teacher_Budget_Planner.xlsx
+++ b/templates/Teacher_Budget_Planner.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Monthly Budget" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Classroom Spending" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Summer Planner" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Salary Comparison" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Instructions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Budget" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classroom Spending" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summer Planner" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Salary Comparison" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -866,7 +866,7 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Subscriptions (Netflix, Spotify, etc.)</t>
+          <t>Subscriptions (streaming service, music subscription, etc.)</t>
         </is>
       </c>
       <c r="B21" s="6" t="n">
@@ -1042,7 +1042,7 @@
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>Expo markers (bulk)</t>
+          <t>Dry-erase markers (bulk)</t>
         </is>
       </c>
       <c r="C2" s="14" t="inlineStr">
@@ -1166,7 +1166,7 @@
       </c>
       <c r="G5" s="16" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Online retailer</t>
         </is>
       </c>
     </row>
@@ -1264,7 +1264,7 @@
       </c>
       <c r="G8" s="14" t="inlineStr">
         <is>
-          <t>Dollar Tree</t>
+          <t>Dollar store</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>Scholastic book order (class set)</t>
+          <t>Book order (class set)</t>
         </is>
       </c>
       <c r="C9" s="16" t="inlineStr">

</xml_diff>